<commit_message>
Add synthetic public-demo screenshots and capture workflow
</commit_message>
<xml_diff>
--- a/data/synthetic/synthetic_comparables.xlsx
+++ b/data/synthetic/synthetic_comparables.xlsx
@@ -610,7 +610,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Demo Pharma Distribution GmbH</t>
+          <t>Demo Comparable 01 GmbH</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -718,7 +718,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Nordic Rx Wholesale AB</t>
+          <t>Demo Comparable 02 AB</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -826,7 +826,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Alpine Medicines Trading AG</t>
+          <t>Demo Comparable 03 AG</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -934,7 +934,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Iberia Pharma Supply SL</t>
+          <t>Demo Comparable 04 SL</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1042,7 +1042,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Baltic Health Distribution OÜ</t>
+          <t>Demo Comparable 05 OU</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1150,7 +1150,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Benelux Medicines Wholesale BV</t>
+          <t>Demo Comparable 06 BV</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1258,7 +1258,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Adriatic Pharma Trade SRL</t>
+          <t>Demo Comparable 07 SRL</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1366,7 +1366,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Central Europe Rx Sp zoo</t>
+          <t>Demo Comparable 08 Sp zoo</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1474,7 +1474,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Lusitania Pharma Logistics SA</t>
+          <t>Demo Comparable 09 SA</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1582,7 +1582,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Danube Healthcare Wholesale Kft</t>
+          <t>Demo Comparable 10 Kft</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">

</xml_diff>